<commit_message>
Pet-Study Models complete, update to many graphics also for the defense
Major update.
</commit_message>
<xml_diff>
--- a/Output/Acute Bout/Tables/t1_biomarkers.xlsx
+++ b/Output/Acute Bout/Tables/t1_biomarkers.xlsx
@@ -459,39 +459,39 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>7.62 (0.472)</t>
+          <t>7.62 (0.47)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.74 (0.842)</t>
+          <t>7.74 (0.84)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7.68 (0.674)</t>
+          <t>7.68 (0.67)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7.45 [7.30, 7.93]</t>
+          <t>7.45 (6.70, 8.50)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7.80 [7.45, 8.15]</t>
+          <t>7.80 (6.00, 10.00)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7.70 [7.30, 8.10]</t>
+          <t>7.70 (6.00, 10.00)</t>
         </is>
       </c>
     </row>
@@ -527,22 +527,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4.45 [4.00, 4.90]</t>
+          <t>4.45 (2.00, 8.60)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4.20 [3.40, 5.40]</t>
+          <t>4.20 (2.90, 9.50)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>4.40 [3.75, 5.05]</t>
+          <t>4.40 (2.00, 9.50)</t>
         </is>
       </c>
     </row>
@@ -561,39 +561,39 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>254 (70.7)</t>
+          <t>253.75 (70.66)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>252 (69.3)</t>
+          <t>252.09 (69.28)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>253 (69.2)</t>
+          <t>252.94 (69.23)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>238 [215, 273]</t>
+          <t>237.50 (125.00, 406.00)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>235 [210, 281]</t>
+          <t>235.00 (161.00, 460.00)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>235 [211, 281]</t>
+          <t>235.00 (125.00, 460.00)</t>
         </is>
       </c>
     </row>
@@ -612,39 +612,39 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1.23 (0.407)</t>
+          <t>1.23 (0.41)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.42 (0.473)</t>
+          <t>1.42 (0.47)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.33 (0.446)</t>
+          <t>1.33 (0.45)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1.20 [0.905, 1.52]</t>
+          <t>1.20 (0.65, 1.98)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.45 [1.07, 1.63]</t>
+          <t>1.45 (0.66, 2.54)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.34 [0.950, 1.57]</t>
+          <t>1.34 (0.65, 2.54)</t>
         </is>
       </c>
     </row>
@@ -663,39 +663,39 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>71.4 (54.8)</t>
+          <t>71.43 (54.76)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>124 (128)</t>
+          <t>124.27 (127.62)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>97.3 (99.9)</t>
+          <t>97.27 (99.93)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>54.0 [29.5, 89.0]</t>
+          <t>54.00 (11.00, 194.00)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>70.0 [37.8, 187]</t>
+          <t>70.00 (11.00, 518.00)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>66.0 [34.0, 121]</t>
+          <t>66.00 (11.00, 518.00)</t>
         </is>
       </c>
     </row>
@@ -736,39 +736,39 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>69.5 (14.1)</t>
+          <t>69.46 (14.14)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>68.5 (13.8)</t>
+          <t>68.52 (13.83)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>69.0 (13.8)</t>
+          <t>69.00 (13.85)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>70.0 [59.0, 75.5]</t>
+          <t>70.00 (43.00, 102.00)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>68.0 [58.5, 76.0]</t>
+          <t>68.00 (40.00, 94.00)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>69.0 [59.0, 76.0]</t>
+          <t>69.00 (40.00, 102.00)</t>
         </is>
       </c>
     </row>
@@ -787,39 +787,39 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0.124 (0.107)</t>
+          <t>0.12 (0.11)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.163 (0.103)</t>
+          <t>0.16 (0.10)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.143 (0.105)</t>
+          <t>0.14 (0.11)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0.100 [0.0560, 0.160]</t>
+          <t>0.10 (0.00, 0.39)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.145 [0.0808, 0.220]</t>
+          <t>0.15 (0.02, 0.35)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.100 [0.0760, 0.220]</t>
+          <t>0.10 (0.00, 0.39)</t>
         </is>
       </c>
     </row>
@@ -860,39 +860,39 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0.876 (0.322)</t>
+          <t>0.88 (0.32)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.11 (0.354)</t>
+          <t>1.11 (0.35)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.987 (0.353)</t>
+          <t>0.99 (0.35)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0.720 [0.660, 1.00]</t>
+          <t>0.72 (0.48, 1.60)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1.10 [0.860, 1.40]</t>
+          <t>1.10 (0.49, 1.80)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.915 [0.718, 1.25]</t>
+          <t>0.92 (0.48, 1.80)</t>
         </is>
       </c>
     </row>
@@ -933,39 +933,39 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0.0949 (0.0557)</t>
+          <t>0.09 (0.06)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.119 (0.0944)</t>
+          <t>0.12 (0.09)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0.107 (0.0768)</t>
+          <t>0.11 (0.08)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0.0940 [0.0495, 0.128]</t>
+          <t>0.09 (0.02, 0.22)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.110 [0.0900, 0.130]</t>
+          <t>0.11 (0.03, 0.45)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.100 [0.0585, 0.130]</t>
+          <t>0.10 (0.02, 0.45)</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0.747 (NA)</t>
+          <t>0.75 (NA)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1016,29 +1016,29 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.747 (NA)</t>
+          <t>0.75 (NA)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0.747 [0.747, 0.747]</t>
+          <t>0.75 (0.75, 0.75)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NA [NA, NA]</t>
+          <t>NA (NA, NA)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0.747 [0.747, 0.747]</t>
+          <t>0.75 (0.75, 0.75)</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0.0890 (NA)</t>
+          <t>0.09 (NA)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1089,29 +1089,29 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0.0890 (NA)</t>
+          <t>0.09 (NA)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0.0890 [0.0890, 0.0890]</t>
+          <t>0.09 (0.09, 0.09)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>NA [NA, NA]</t>
+          <t>NA (NA, NA)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.0890 [0.0890, 0.0890]</t>
+          <t>0.09 (0.09, 0.09)</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1169,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1.41 [0.623, 3.33]</t>
+          <t>1.41 (0.07, 7.37)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1.47 [0.504, 6.04]</t>
+          <t>1.47 (0.02, 15.21)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>1.41 [0.508, 4.56]</t>
+          <t>1.41 (0.02, 15.21)</t>
         </is>
       </c>
     </row>
@@ -1225,39 +1225,39 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0.151 (0.106)</t>
+          <t>0.15 (0.11)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.107 (0.0557)</t>
+          <t>0.11 (0.06)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0.127 (0.0834)</t>
+          <t>0.13 (0.08)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0.123 [0.0821, 0.186]</t>
+          <t>0.12 (0.04, 0.37)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.0909 [0.0763, 0.164]</t>
+          <t>0.09 (0.03, 0.19)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.119 [0.0763, 0.166]</t>
+          <t>0.12 (0.03, 0.37)</t>
         </is>
       </c>
     </row>
@@ -1298,39 +1298,39 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>294 (227)</t>
+          <t>293.89 (226.89)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>168 (112)</t>
+          <t>168.48 (111.75)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>228 (185)</t>
+          <t>228.33 (185.33)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>221 [147, 310]</t>
+          <t>221.46 (123.39, 939.05)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>140 [100, 221]</t>
+          <t>140.12 (21.89, 490.53)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>176 [125, 261]</t>
+          <t>176.26 (21.89, 939.05)</t>
         </is>
       </c>
     </row>
@@ -1371,39 +1371,39 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0.232 (0.102)</t>
+          <t>0.23 (0.10)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.277 (0.126)</t>
+          <t>0.28 (0.13)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.256 (0.116)</t>
+          <t>0.26 (0.12)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0.226 [0.168, 0.303]</t>
+          <t>0.23 (0.07, 0.40)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.242 [0.186, 0.377]</t>
+          <t>0.24 (0.11, 0.49)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0.230 [0.179, 0.359]</t>
+          <t>0.23 (0.07, 0.49)</t>
         </is>
       </c>
     </row>
@@ -1444,39 +1444,39 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0.946 (0.883)</t>
+          <t>0.95 (0.88)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1.02 (0.776)</t>
+          <t>1.02 (0.78)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0.981 (0.824)</t>
+          <t>0.98 (0.82)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0.639 [0.539, 0.903]</t>
+          <t>0.64 (0.19, 4.47)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.776 [0.441, 1.44]</t>
+          <t>0.78 (0.35, 3.06)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>0.688 [0.516, 1.11]</t>
+          <t>0.69 (0.19, 4.47)</t>
         </is>
       </c>
     </row>
@@ -1517,39 +1517,39 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>57400 (22100)</t>
+          <t>57408.40 (22058.21)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>53300 (14100)</t>
+          <t>53251.36 (14134.16)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>55300 (18400)</t>
+          <t>55329.88 (18438.00)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>51400 [40400, 71000]</t>
+          <t>51353.19 (31298.35, 110315.04)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>53400 [42700, 59200]</t>
+          <t>53367.83 (23273.96, 82777.54)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>52900 [40300, 59700]</t>
+          <t>52864.39 (23273.96, 110315.04)</t>
         </is>
       </c>
     </row>
@@ -1590,39 +1590,39 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>0.400 (0.199)</t>
+          <t>0.40 (0.20)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.471 (0.469)</t>
+          <t>0.47 (0.47)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.436 (0.361)</t>
+          <t>0.44 (0.36)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0.367 [0.234, 0.516]</t>
+          <t>0.37 (0.10, 0.80)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.263 [0.203, 0.356]</t>
+          <t>0.26 (0.15, 1.70)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.310 [0.216, 0.502]</t>
+          <t>0.31 (0.10, 1.70)</t>
         </is>
       </c>
     </row>
@@ -1668,34 +1668,34 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>6.17 (15.4)</t>
+          <t>6.17 (15.45)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.07 (12.9)</t>
+          <t>5.07 (12.94)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>1.56 [1.21, 2.59]</t>
+          <t>1.56 (0.81, 48.17)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>1.50 [1.11, 1.87]</t>
+          <t>1.50 (0.44, 55.95)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>1.51 [1.15, 2.17]</t>
+          <t>1.51 (0.44, 55.95)</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>0.811 (0.997)</t>
+          <t>0.81 (1.00)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1753,22 +1753,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>0.583 [0.198, 0.631]</t>
+          <t>0.58 (0.10, 2.54)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>3.12 [3.12, 3.12]</t>
+          <t>3.12 (3.12, 3.12)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.607 [0.294, 2.07]</t>
+          <t>0.61 (0.10, 3.12)</t>
         </is>
       </c>
     </row>
@@ -1809,39 +1809,39 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>16.0 (15.9)</t>
+          <t>16.01 (15.88)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>13.2 (14.0)</t>
+          <t>13.16 (13.99)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>14.6 (14.8)</t>
+          <t>14.55 (14.84)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Median [Q1, Q3]</t>
+          <t xml:space="preserve">  Median (Min, Max)</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>8.58 [5.78, 19.7]</t>
+          <t>8.58 (1.28, 54.97)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>7.09 [5.21, 17.1]</t>
+          <t>7.09 (1.45, 59.55)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>8.39 [5.54, 19.3]</t>
+          <t>8.39 (1.28, 59.55)</t>
         </is>
       </c>
     </row>

</xml_diff>